<commit_message>
MediBec: S2 and S8 scored AV:L; reference totals 84,305 / 41,023
The representative weakness of S2 (ransomware) and S8 (detection gap) is a
malicious e-mailed document opened locally, which the FIRST CVSS v4.0 user
guide scores as Local: S2 9.4 -> 9.3, S8 9.3 -> 9.2. Recomputed with
crg_calc: total estimated 84,305 and residual 41,023 (was 84,491 / 41,104);
no verdict changes (12 above, 11 approximately at, 7 below).

- data.py writes data.json; data30.json, medibec30.json and budget.json
  regenerated from the sources
- retired markers replaced with Analytical estimate / Information gap in
  every builder; 'CyberRiskGuardian KRIs' headers renamed risk indices
- all seven deliverables rebuilt (openpyxl, docx-js), workbooks
  recalculated with LibreOffice: 0 formula errors, totals equal crg_calc

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A2TtsRJov8uxPoHCkXTh3x
</commit_message>
<xml_diff>
--- a/examples/medibec/deliverables/MediBec_CyberRiskGuardian_Workbook.xlsx
+++ b/examples/medibec/deliverables/MediBec_CyberRiskGuardian_Workbook.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId3"/>
@@ -775,7 +775,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Representative weakness: malicious macro document leading to code execution (initial vector in E6). AV:N delivered by e-mail; AC:L; AT:N; PR:N; UI:P user opens the document; VC/VI/VA:H on the workstation; SC/SI/SA:H because EHR and clinic systems are subsequently affected. CVSS describes the entry weakness only, not the enterprise impact.</t>
+          <t xml:space="preserve">Representative weakness: malicious macro document leading to code execution (initial vector in E6). AV:L: the document is delivered by e-mail but opened and executed locally on the workstation (FIRST CVSS v4.0 user guide scores malicious documents as Local whatever the delivery channel); AC:L; AT:N; PR:N; UI:P user opens the document; VC/VI/VA:H on the workstation; SC/SI/SA:H because EHR and clinic systems are subsequently affected. CVSS describes the entry weakness only, not the enterprise impa</t>
         </r>
       </text>
     </comment>
@@ -847,7 +847,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Limited applicability: a detection gap is a control weakness, not a vulnerability. Representative weakness for the workbook: the undetected initial code-execution vector (macro/PowerShell, E6). Do not interpret the score as the severity of the detection gap.</t>
+          <t xml:space="preserve">Limited applicability: a detection gap is a control weakness, not a vulnerability. Representative weakness for the workbook: the undetected initial code-execution vector (macro/PowerShell, E6), scored AV:L because the e-mailed document is opened and executed locally (FIRST CVSS v4.0 user guide). Do not interpret the score as the severity of the detection gap.</t>
         </r>
       </text>
     </comment>
@@ -891,7 +891,7 @@
     <t xml:space="preserve">Source: MediBec Business Case v2.0b (fictional teaching case, M.-A. Leger) and CyberRiskGuardian Excel Guide v1.0c formulas.</t>
   </si>
   <si>
-    <t xml:space="preserve">All parameter values, CVSS vectors, costs and reductions are ANALYST ESTIMATES - VALIDATION REQUIRED. Scores are relative decision-support indicators, not loss predictions.</t>
+    <t xml:space="preserve">All parameter values, CVSS vectors, costs and reductions are analytical estimates (Analytical estimate — validation required). Scores are relative decision-support indicators, not loss predictions.</t>
   </si>
   <si>
     <t xml:space="preserve">Colour legend:  blue text = input you may edit  |  black = formula  |  green = link to another sheet  |  yellow fill = key assumption.</t>
@@ -942,7 +942,7 @@
     <t xml:space="preserve">How to use: change blue cells on Parameters / Inputs / Portfolio, then recalculate (Formulas &gt; Calculate Now if manual).</t>
   </si>
   <si>
-    <t xml:space="preserve">Analyse - CyberRiskGuardian KRIs (Excel Guide v1.0c formulas)</t>
+    <t xml:space="preserve">Analyse - CyberRiskGuardian risk indices (Excel Guide v1.0c formulas)</t>
   </si>
   <si>
     <t xml:space="preserve">Green = linked from Inputs / Portfolio / Parameters; black = formula.</t>
@@ -1035,10 +1035,10 @@
     <t xml:space="preserve">Source / note</t>
   </si>
   <si>
-    <t xml:space="preserve">Risk appetite (analyst estimate)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyst estimate - validation required. Case states 0.40 normalized tolerance; see report s.4.</t>
+    <t xml:space="preserve">Risk appetite (analytical estimate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analytical estimate — validation required. Case states 0.40 normalized tolerance; see report s.4.</t>
   </si>
   <si>
     <t xml:space="preserve">Multiplication factor</t>
@@ -1077,7 +1077,7 @@
     <t xml:space="preserve">Case escalation - Board acceptance threshold</t>
   </si>
   <si>
-    <t xml:space="preserve">Scenario inputs (0-1 scale unless stated) - Analyst estimates, validation required</t>
+    <t xml:space="preserve">Scenario inputs (0-1 scale unless stated) - Analytical estimate — validation required</t>
   </si>
   <si>
     <t xml:space="preserve">CVSS v4.0 vector</t>
@@ -1125,7 +1125,7 @@
     <t xml:space="preserve">Ransomware disrupting EHR access and clinic operations across the network</t>
   </si>
   <si>
-    <t xml:space="preserve">CVSS:4.0/AV:N/AC:L/AT:N/PR:N/UI:P/VC:H/VI:H/VA:H/SC:H/SI:H/SA:H</t>
+    <t xml:space="preserve">CVSS:4.0/AV:L/AC:L/AT:N/PR:N/UI:P/VC:H/VI:H/VA:H/SC:H/SI:H/SA:H</t>
   </si>
   <si>
     <t xml:space="preserve">S3</t>
@@ -1179,7 +1179,7 @@
     <t xml:space="preserve">Detection and response gaps allow an intrusion to persist and escalate</t>
   </si>
   <si>
-    <t xml:space="preserve">CVSS:4.0/AV:N/AC:L/AT:N/PR:N/UI:P/VC:H/VI:H/VA:L/SC:H/SI:L/SA:L</t>
+    <t xml:space="preserve">CVSS:4.0/AV:L/AC:L/AT:N/PR:N/UI:P/VC:H/VI:H/VA:L/SC:H/SI:L/SA:L</t>
   </si>
   <si>
     <t xml:space="preserve">S9</t>
@@ -1464,7 +1464,7 @@
     <t xml:space="preserve">Allocation assumption: each initiative's Year-1 cost is split equally across the scenarios it addresses, so shared controls are never charged in full to several scenarios.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cyber-insurance premium is excluded (Evidence gap - broker quotation required).</t>
+    <t xml:space="preserve">Cyber-insurance premium is excluded (Information gap — organizational validation required: broker quotation required).</t>
   </si>
   <si>
     <t xml:space="preserve">Sensitivity - lower / central / higher cases</t>
@@ -1590,7 +1590,7 @@
     <t xml:space="preserve">Cybercriminal (initial-access broker or ransomware affiliate).</t>
   </si>
   <si>
-    <t xml:space="preserve">Push-based MFA without number matching or phishing resistance (E6 - validate); No evidence of conditional access (geo/device) policies; Internet-sourced macro documents reach users (E6); Awareness programme maturity unknown (Evidence gap)</t>
+    <t xml:space="preserve">Push-based MFA without number matching or phishing resistance (E6 - validate); No evidence of conditional access (geo/device) policies; Internet-sourced macro documents reach users (E6); Awareness programme maturity unknown (Information gap)</t>
   </si>
   <si>
     <t xml:space="preserve">Email filtering / antimalware (E2 - effectiveness unknown); MFA push on remote access (E6); EDR alerting (E6 - triage weak)</t>
@@ -1620,7 +1620,7 @@
     <t xml:space="preserve">Ransomware-as-a-service affiliate (double extortion).</t>
   </si>
   <si>
-    <t xml:space="preserve">Macro execution and weak alert triage (E6); Segmentation between clinics, servers and backups not evidenced (E2, E7); Privileged credential hygiene unknown (Evidence gap); Clinic downtime procedures untested (E7)</t>
+    <t xml:space="preserve">Macro execution and weak alert triage (E6); Segmentation between clinics, servers and backups not evidenced (E2, E7); Privileged credential hygiene unknown (Information gap); Clinic downtime procedures untested (E7)</t>
   </si>
   <si>
     <t xml:space="preserve">Firewalls, IDS/IPS, antimalware (E2); EDR (E6); On-site and off-site backups (E2 - isolation and testing unknown); Incident command structure defined (E6 - untested)</t>
@@ -1638,7 +1638,7 @@
     <t xml:space="preserve">0-24 months</t>
   </si>
   <si>
-    <t xml:space="preserve">Representative weakness: malicious macro document leading to code execution (initial vector in E6). AV:N delivered by e-mail; AC:L; AT:N; PR:N; UI:P user opens the document; VC/VI/VA:H on the workstation; SC/SI/SA:H because EHR and clinic systems are subsequently affected. CVSS describes the entry weakness only, not the enterprise impact.</t>
+    <t xml:space="preserve">Representative weakness: malicious macro document leading to code execution (initial vector in E6). AV:L: the document is delivered by e-mail but opened and executed locally on the workstation (FIRST CVSS v4.0 user guide scores malicious documents as Local whatever the delivery channel); AC:L; AT:N; PR:N; UI:P user opens the document; VC/VI/VA:H on the workstation; SC/SI/SA:H because EHR and clinic systems are subsequently affected. CVSS describes the entry weakness only, not the enterprise impact.</t>
   </si>
   <si>
     <t xml:space="preserve">MED-CYR-07</t>
@@ -1734,7 +1734,7 @@
     <t xml:space="preserve">Cybercriminal / state-linked actor using public exploits.</t>
   </si>
   <si>
-    <t xml:space="preserve">Patch SLAs and exception governance not evidenced (E7); Incomplete asset inventory (E4); Possible end-of-life systems (Evidence gap)</t>
+    <t xml:space="preserve">Patch SLAs and exception governance not evidenced (E7); Incomplete asset inventory (E4); Possible end-of-life systems (Information gap)</t>
   </si>
   <si>
     <t xml:space="preserve">Firewalls, IDS/IPS (E2); Antimalware (E2)</t>
@@ -1803,7 +1803,7 @@
     <t xml:space="preserve">I01, I03, I11, I12</t>
   </si>
   <si>
-    <t xml:space="preserve">Limited applicability: a detection gap is a control weakness, not a vulnerability. Representative weakness for the workbook: the undetected initial code-execution vector (macro/PowerShell, E6). Do not interpret the score as the severity of the detection gap.</t>
+    <t xml:space="preserve">Limited applicability: a detection gap is a control weakness, not a vulnerability. Representative weakness for the workbook: the undetected initial code-execution vector (macro/PowerShell, E6), scored AV:L because the e-mailed document is opened and executed locally (FIRST CVSS v4.0 user guide). Do not interpret the score as the severity of the detection gap.</t>
   </si>
   <si>
     <t xml:space="preserve">MED-CYR-14</t>
@@ -2760,7 +2760,7 @@
     <t xml:space="preserve">Methodology</t>
   </si>
   <si>
-    <t xml:space="preserve">Authoritative KRI formulas; CVSS v4.0; multiplication factor 1,000 in worked example; reductions must stay within 0-1.</t>
+    <t xml:space="preserve">Authoritative risk-index formulas; CVSS v4.0; multiplication factor 1,000 in worked example; reductions must stay within 0-1.</t>
   </si>
   <si>
     <t xml:space="preserve">E11</t>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">Inputs!J5</f>
-        <v>9.4</v>
+        <v>9.3</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">Inputs!E5</f>
@@ -4361,11 +4361,11 @@
       </c>
       <c r="L6" s="9" t="n">
         <f aca="false">C6*D6*E6*((F6+G6)/2)*H6/I6*K6</f>
-        <v>7893.48214285714</v>
+        <v>7809.50892857143</v>
       </c>
       <c r="M6" s="9" t="n">
         <f aca="false">C6*D6*E6*J6*H6/I6*K6</f>
-        <v>2870.35714285714</v>
+        <v>2839.82142857143</v>
       </c>
       <c r="N6" s="10" t="n">
         <f aca="false">L6/M6</f>
@@ -4385,11 +4385,11 @@
       </c>
       <c r="R6" s="9" t="n">
         <f aca="false">L6*P6*Q6</f>
-        <v>4440.08370535714</v>
+        <v>4392.84877232143</v>
       </c>
       <c r="S6" s="9" t="n">
         <f aca="false">L6-R6</f>
-        <v>3453.3984375</v>
+        <v>3416.66015625</v>
       </c>
       <c r="T6" s="10" t="n">
         <f aca="false">S6/M6</f>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="V6" s="10" t="n">
         <f aca="false">IF(O6=0,0,(L6-S6)/O6*1000)</f>
-        <v>7.57837158130368</v>
+        <v>7.49775060703449</v>
       </c>
       <c r="W6" s="12" t="str">
         <f aca="false">IF(AND(P6&gt;=0,P6&lt;=1,Q6&gt;=0,Q6&lt;=1),"OK","CHECK")</f>
@@ -4897,7 +4897,7 @@
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">Inputs!J11</f>
-        <v>9.3</v>
+        <v>9.2</v>
       </c>
       <c r="F12" s="6" t="n">
         <f aca="false">Inputs!E11</f>
@@ -4925,11 +4925,11 @@
       </c>
       <c r="L12" s="9" t="n">
         <f aca="false">C12*D12*E12*((F12+G12)/2)*H12/I12*K12</f>
-        <v>9486</v>
+        <v>9384</v>
       </c>
       <c r="M12" s="9" t="n">
         <f aca="false">C12*D12*E12*J12*H12/I12*K12</f>
-        <v>3794.4</v>
+        <v>3753.6</v>
       </c>
       <c r="N12" s="10" t="n">
         <f aca="false">L12/M12</f>
@@ -4949,11 +4949,11 @@
       </c>
       <c r="R12" s="9" t="n">
         <f aca="false">L12*P12*Q12</f>
-        <v>5312.16</v>
+        <v>5255.04</v>
       </c>
       <c r="S12" s="9" t="n">
         <f aca="false">L12-R12</f>
-        <v>4173.84</v>
+        <v>4128.96</v>
       </c>
       <c r="T12" s="10" t="n">
         <f aca="false">S12/M12</f>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="V12" s="10" t="n">
         <f aca="false">IF(O12=0,0,(L12-S12)/O12*1000)</f>
-        <v>25.4305531914894</v>
+        <v>25.1571063829787</v>
       </c>
       <c r="W12" s="12" t="str">
         <f aca="false">IF(AND(P12&gt;=0,P12&lt;=1,Q12&gt;=0,Q12&lt;=1),"OK","CHECK")</f>
@@ -5166,11 +5166,11 @@
       </c>
       <c r="L15" s="14" t="n">
         <f aca="false">SUM(L5:L14)</f>
-        <v>50492.1348214286</v>
+        <v>50306.1616071429</v>
       </c>
       <c r="M15" s="14" t="n">
         <f aca="false">SUM(M5:M14)</f>
-        <v>20507.8888392857</v>
+        <v>20436.553125</v>
       </c>
       <c r="O15" s="15" t="n">
         <f aca="false">SUM(O5:O14)</f>
@@ -5178,19 +5178,19 @@
       </c>
       <c r="R15" s="14" t="n">
         <f aca="false">SUM(R5:R14)</f>
-        <v>27688.1059754464</v>
+        <v>27583.7510424107</v>
       </c>
       <c r="S15" s="14" t="n">
         <f aca="false">SUM(S5:S14)</f>
-        <v>22804.0288459821</v>
+        <v>22722.4105647321</v>
       </c>
       <c r="T15" s="16" t="n">
         <f aca="false">S15/M15</f>
-        <v>1.11196374354721</v>
+        <v>1.11185141769019</v>
       </c>
       <c r="V15" s="16" t="n">
         <f aca="false">(L15-S15)/O15*1000</f>
-        <v>7.16195188190544</v>
+        <v>7.13495888318953</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5516,7 +5516,7 @@
         <v>81</v>
       </c>
       <c r="J5" s="21" t="n">
-        <v>9.4</v>
+        <v>9.3</v>
       </c>
       <c r="K5" s="20" t="n">
         <v>0.75</v>
@@ -5852,7 +5852,7 @@
         <v>99</v>
       </c>
       <c r="J11" s="21" t="n">
-        <v>9.3</v>
+        <v>9.2</v>
       </c>
       <c r="K11" s="20" t="n">
         <v>0.7</v>
@@ -7267,7 +7267,7 @@
       </c>
       <c r="J5" s="7" t="n">
         <f aca="false">Inputs!J5</f>
-        <v>9.4</v>
+        <v>9.3</v>
       </c>
       <c r="K5" s="10" t="n">
         <f aca="false">MAX(0.05,MIN(0.99,Inputs!K5-C5))</f>
@@ -7279,15 +7279,15 @@
       </c>
       <c r="M5" s="9" t="n">
         <f aca="false">D5*E5*J5*((F5+G5)/2)*I5/H5*Parameters!$B$5</f>
-        <v>3740.67777777778</v>
+        <v>3700.88333333333</v>
       </c>
       <c r="N5" s="9" t="n">
         <f aca="false">D5*E5*J5*Parameters!$B$4*I5/H5*Parameters!$B$5</f>
-        <v>1547.86666666667</v>
+        <v>1531.4</v>
       </c>
       <c r="O5" s="9" t="n">
         <f aca="false">M5-M5*K5*L5</f>
-        <v>1038.03808333333</v>
+        <v>1026.995125</v>
       </c>
       <c r="P5" s="10" t="n">
         <f aca="false">O5/N5</f>
@@ -7335,7 +7335,7 @@
       </c>
       <c r="J6" s="7" t="n">
         <f aca="false">Inputs!J5</f>
-        <v>9.4</v>
+        <v>9.3</v>
       </c>
       <c r="K6" s="10" t="n">
         <f aca="false">MAX(0.05,MIN(0.99,Inputs!K5-C6))</f>
@@ -7347,15 +7347,15 @@
       </c>
       <c r="M6" s="9" t="n">
         <f aca="false">D6*E6*J6*((F6+G6)/2)*I6/H6*Parameters!$B$5</f>
-        <v>7893.48214285714</v>
+        <v>7809.50892857143</v>
       </c>
       <c r="N6" s="9" t="n">
         <f aca="false">D6*E6*J6*Parameters!$B$4*I6/H6*Parameters!$B$5</f>
-        <v>2870.35714285714</v>
+        <v>2839.82142857143</v>
       </c>
       <c r="O6" s="9" t="n">
         <f aca="false">M6-M6*K6*L6</f>
-        <v>3453.3984375</v>
+        <v>3416.66015625</v>
       </c>
       <c r="P6" s="10" t="n">
         <f aca="false">O6/N6</f>
@@ -7403,7 +7403,7 @@
       </c>
       <c r="J7" s="7" t="n">
         <f aca="false">Inputs!J5</f>
-        <v>9.4</v>
+        <v>9.3</v>
       </c>
       <c r="K7" s="10" t="n">
         <f aca="false">MAX(0.05,MIN(0.99,Inputs!K5-C7))</f>
@@ -7415,15 +7415,15 @@
       </c>
       <c r="M7" s="9" t="n">
         <f aca="false">D7*E7*J7*((F7+G7)/2)*I7/H7*Parameters!$B$5</f>
-        <v>16304.394</v>
+        <v>16130.943</v>
       </c>
       <c r="N7" s="9" t="n">
         <f aca="false">D7*E7*J7*Parameters!$B$4*I7/H7*Parameters!$B$5</f>
-        <v>5465.16</v>
+        <v>5407.02</v>
       </c>
       <c r="O7" s="9" t="n">
         <f aca="false">M7-M7*K7*L7</f>
-        <v>9415.787535</v>
+        <v>9315.6195825</v>
       </c>
       <c r="P7" s="10" t="n">
         <f aca="false">O7/N7</f>
@@ -8083,7 +8083,7 @@
       </c>
       <c r="J17" s="7" t="n">
         <f aca="false">Inputs!J11</f>
-        <v>9.3</v>
+        <v>9.2</v>
       </c>
       <c r="K17" s="10" t="n">
         <f aca="false">MAX(0.05,MIN(0.99,Inputs!K11-C17))</f>
@@ -8095,15 +8095,15 @@
       </c>
       <c r="M17" s="9" t="n">
         <f aca="false">D17*E17*J17*((F17+G17)/2)*I17/H17*Parameters!$B$5</f>
-        <v>4495.96875</v>
+        <v>4447.625</v>
       </c>
       <c r="N17" s="9" t="n">
         <f aca="false">D17*E17*J17*Parameters!$B$4*I17/H17*Parameters!$B$5</f>
-        <v>2075.0625</v>
+        <v>2052.75</v>
       </c>
       <c r="O17" s="9" t="n">
         <f aca="false">M17-M17*K17*L17</f>
-        <v>1258.87125</v>
+        <v>1245.335</v>
       </c>
       <c r="P17" s="10" t="n">
         <f aca="false">O17/N17</f>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="J18" s="7" t="n">
         <f aca="false">Inputs!J11</f>
-        <v>9.3</v>
+        <v>9.2</v>
       </c>
       <c r="K18" s="10" t="n">
         <f aca="false">MAX(0.05,MIN(0.99,Inputs!K11-C18))</f>
@@ -8163,15 +8163,15 @@
       </c>
       <c r="M18" s="9" t="n">
         <f aca="false">D18*E18*J18*((F18+G18)/2)*I18/H18*Parameters!$B$5</f>
-        <v>9486</v>
+        <v>9384</v>
       </c>
       <c r="N18" s="9" t="n">
         <f aca="false">D18*E18*J18*Parameters!$B$4*I18/H18*Parameters!$B$5</f>
-        <v>3794.4</v>
+        <v>3753.6</v>
       </c>
       <c r="O18" s="9" t="n">
         <f aca="false">M18-M18*K18*L18</f>
-        <v>4173.84</v>
+        <v>4128.96</v>
       </c>
       <c r="P18" s="10" t="n">
         <f aca="false">O18/N18</f>
@@ -8219,7 +8219,7 @@
       </c>
       <c r="J19" s="7" t="n">
         <f aca="false">Inputs!J11</f>
-        <v>9.3</v>
+        <v>9.2</v>
       </c>
       <c r="K19" s="10" t="n">
         <f aca="false">MAX(0.05,MIN(0.99,Inputs!K11-C19))</f>
@@ -8231,15 +8231,15 @@
       </c>
       <c r="M19" s="9" t="n">
         <f aca="false">D19*E19*J19*((F19+G19)/2)*I19/H19*Parameters!$B$5</f>
-        <v>21041.13375</v>
+        <v>20814.885</v>
       </c>
       <c r="N19" s="9" t="n">
         <f aca="false">D19*E19*J19*Parameters!$B$4*I19/H19*Parameters!$B$5</f>
-        <v>7470.225</v>
+        <v>7389.9</v>
       </c>
       <c r="O19" s="9" t="n">
         <f aca="false">M19-M19*K19*L19</f>
-        <v>12203.857575</v>
+        <v>12072.6333</v>
       </c>
       <c r="P19" s="10" t="n">
         <f aca="false">O19/N19</f>
@@ -9041,7 +9041,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
         <v>79</v>
       </c>
@@ -9269,7 +9269,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
         <v>97</v>
       </c>

</xml_diff>